<commit_message>
refactor: rephrase columns - 'type' -> 'driver', and 'f/f (form factor)' -> 'style'
</commit_message>
<xml_diff>
--- a/presets/letter/TEMPLATE.xlsx
+++ b/presets/letter/TEMPLATE.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'List'!$A$1:$N$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'List'!$A$1:$O$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -740,7 +740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -749,7 +749,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="58" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="58" customWidth="1" min="8" max="8"/>
     <col width="58" customWidth="1" min="9" max="9"/>
     <col width="58" customWidth="1" min="10" max="10"/>
@@ -757,6 +757,7 @@
     <col width="58" customWidth="1" min="12" max="12"/>
     <col width="58" customWidth="1" min="13" max="13"/>
     <col width="58" customWidth="1" min="14" max="14"/>
+    <col width="58" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -782,50 +783,55 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Driver</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Style</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Tags</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Pros</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Cons</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Comment_KR</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Pros_KR</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Cons_KR</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Notes_KR</t>
         </is>
@@ -858,47 +864,52 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>IEM</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>Personal Collection, Reference</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Reference sound with a neutral tilt.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Even tonality
 Excellent detail retrieval</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Fit may be shallow for small ears</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Measured with a stock silicone tip.</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>레퍼런스 사운드에 가까운 중립적인 튜닝.</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>고른 음색
 뛰어난 디테일</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>귀가 작으면 착용감이 얕을 수 있음</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>기본 실리콘 팁으로 측정했습니다.</t>
         </is>
@@ -931,41 +942,46 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>IEM</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Warm and forgiving.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Smooth treble</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Soft sub-bass</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>따뜻하고 편안한 소리.</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>부드러운 고음</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>서브베이스가 약함</t>
         </is>
       </c>
-      <c r="N3" s="2" t="n"/>
+      <c r="O3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -992,35 +1008,40 @@
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>IEM</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Not recommended.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Peaky upper midrange
 Poor build quality</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>추천하지 않습니다.</t>
         </is>
       </c>
-      <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>중고음 피크
 낮은 빌드 품질</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n"/>
+      <c r="O4" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N4"/>
+  <autoFilter ref="A1:O4"/>
   <conditionalFormatting sqref="C2:C1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"S"</formula>
@@ -1068,7 +1089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="92" customWidth="1" min="1" max="1"/>
@@ -1311,136 +1332,143 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Type — Hybrid, DD, BA, planar. Becomes a chip and a filter.</t>
+          <t>Driver — Hybrid, DD, BA, planar. Becomes a chip and a filter.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Tags — Comma separated. Shown as pills, and searchable.</t>
+          <t>Style — Open, closed, IEM, earbud. Becomes a chip and a filter.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Comment — The main paragraph.</t>
+          <t>Tags — Comma separated. Shown as pills, and searchable.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Pros — A green block. Alt+Enter for one point per line.</t>
+          <t>Comment — The main paragraph.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Cons — A red block. Alt+Enter for one point per line.</t>
+          <t>Pros — A green block. Alt+Enter for one point per line.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Notes — A muted block, for caveats and measurement remarks.</t>
+          <t>Cons — A red block. Alt+Enter for one point per line.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Comment_KR — Korean text for Comment. Blank falls back to English.</t>
+          <t>Notes — A muted block, for caveats and measurement remarks.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Pros_KR — Korean text for Pros. Blank falls back to English.</t>
+          <t>Comment_KR — Korean text for Comment. Blank falls back to English.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cons_KR — Korean text for Cons. Blank falls back to English.</t>
+          <t>Pros_KR — Korean text for Pros. Blank falls back to English.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>Cons_KR — Korean text for Cons. Blank falls back to English.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>Notes_KR — Korean text for Notes. Blank falls back to English.</t>
         </is>
       </c>
     </row>
-    <row r="34"/>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Line breaks inside a cell are kept. Use Alt+Enter (Option+Enter on a Mac).</t>
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>Publishing this sheet for the page</t>
         </is>
       </c>
     </row>
-    <row r="38"/>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>1. File - Share - Publish to web</t>
-        </is>
-      </c>
-    </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2. In the Link tab, choose this sheet and 'Comma-separated values (.csv)'</t>
+          <t>1. File - Share - Publish to web</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>3. Publish, then copy the URL it gives you</t>
+          <t>2. In the Link tab, choose this sheet and 'Comma-separated values (.csv)'</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>3. Publish, then copy the URL it gives you</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>4. Paste it into ranking-config.js as source.url</t>
         </is>
       </c>
     </row>
-    <row r="43"/>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>Do not rename the header row: ranking-config.js looks the columns up by name.</t>
         </is>
       </c>
     </row>
-    <row r="45"/>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Full guide: https://potatosalad775.github.io/squigRanking/docs/setup/your-sheet/</t>
-        </is>
-      </c>
-    </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" t="inlineStr">
+        <is>
+          <t>Full guide: https://potatosalad775.github.io/squigRanking/docs/setup/your-sheet/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Build a config from a form: https://potatosalad775.github.io/squigRanking/docs/config-editor/</t>
         </is>

</xml_diff>